<commit_message>
[Artikel Promo] - Import Data fixed up prd
</commit_message>
<xml_diff>
--- a/public/upload/template/artikel_promo_template.xlsx
+++ b/public/upload/template/artikel_promo_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\jez_sistem\public\upload\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WINDOWS 10\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC7A026-2E4A-48C8-A74F-CA0BA627EA5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4FE0DF-1519-4DA7-9993-F55A892C5897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,18 +25,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>ARTICLE</t>
+  </si>
+  <si>
+    <t>PROMO</t>
+  </si>
+  <si>
+    <t>STORE</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
   <si>
     <t>BAYAR SATU DAPAT DUA</t>
-  </si>
-  <si>
-    <t>ONLINE MALANG</t>
-  </si>
-  <si>
-    <t>DM</t>
-  </si>
-  <si>
-    <t>SPSARD08</t>
   </si>
   <si>
     <t>JANTASTIC</t>
@@ -45,45 +57,28 @@
     <t>JEZ SURABAYA</t>
   </si>
   <si>
-    <t>OFFLINE STORE</t>
+    <t>JEZ MALANG</t>
   </si>
   <si>
-    <t>article_id</t>
-  </si>
-  <si>
-    <t>store</t>
-  </si>
-  <si>
-    <t>promo_name</t>
-  </si>
-  <si>
-    <t>start_date</t>
-  </si>
-  <si>
-    <t>end_date</t>
-  </si>
-  <si>
-    <t>promo_type</t>
-  </si>
-  <si>
-    <t>promo_disc</t>
-  </si>
-  <si>
-    <t>promo_note</t>
+    <t>SPE1010202</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-  </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -115,20 +110,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -341,105 +335,92 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:G1000"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="26" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" customWidth="1"/>
+    <col min="4" max="5" width="11.33203125" customWidth="1"/>
+    <col min="6" max="24" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>11040090</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3">
+        <v>45653</v>
+      </c>
+      <c r="E2" s="4">
+        <v>45717</v>
+      </c>
+      <c r="F2" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="1"/>
+      <c r="D3" s="4">
+        <v>45931</v>
+      </c>
+      <c r="E3" s="3">
+        <v>45683</v>
+      </c>
+      <c r="F3" s="5">
+        <v>50</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>402251</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="4">
-        <v>45653</v>
-      </c>
-      <c r="E2" s="4">
-        <v>45654</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="2">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="4">
-        <v>45318</v>
-      </c>
-      <c r="E3" s="4">
-        <v>45654</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0.55000000000000004</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1426,6 +1407,6 @@
     <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" r:id="rId1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>